<commit_message>
Fail a metadata import on an empty symphonytheme cell
A band without a symphonytheme value does not render in the default UI. A file that has the column but leaves it empty for some bands is now treated as malformed: the import fails with a message naming those bands, before any metadata is written. A file without the column still imports, with the existing notice, and other empty cells are still skipped.

The empty-cells fixture no longer leaves a theme empty.
</commit_message>
<xml_diff>
--- a/src/test/resources/import/metadata-wellformed-empty-cells-en.xlsx
+++ b/src/test/resources/import/metadata-wellformed-empty-cells-en.xlsx
@@ -54,10 +54,10 @@
     <t>Artificial reef</t>
   </si>
   <si>
+    <t>Habitat</t>
+  </si>
+  <si>
     <t/>
-  </si>
-  <si>
-    <t>This raster intends to show presence of artificial reef structures (i.e. bridges, lighthouses at sea, wind power turbines, wrecks etc.) in Swedish coastal and offshore waters.  The surface area of artificial reefs has not been determined. Data shows only the occurrence of artificial structures that can form artificial reefs with a resolution of 250 x 250 m. A cell value of 0 is equivalent to no presence and a cell value of 100 is equivalent to presence. Underlying data are from several different sources and consist of presence data in the form of shapefiles.</t>
   </si>
   <si>
     <t>3</t>
@@ -293,7 +293,7 @@
         <v>26</v>
       </c>
       <c r="E6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F6" t="s">
         <v>11</v>

</xml_diff>